<commit_message>
content(checklist): agrega sección Pensiones y AFORE (IMSS/ISSSTE) al checklist de discapacidad
Nueva sección 4 con 6 ítems sobre pensión por orfandad, beneficiarios de
AFORE y recursos heredables, en lenguaje cauto YMYL ("conforme a la ley").

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/descargas/checklist-proteccion-hijo-discapacidad.xlsx
+++ b/public/descargas/checklist-proteccion-hijo-discapacidad.xlsx
@@ -543,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -965,7 +965,7 @@
     <row r="42" ht="26" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>4. Fideicomiso o mecanismo de administración</t>
+          <t>4. Pensiones y AFORE (IMSS / ISSSTE)</t>
         </is>
       </c>
       <c r="B42" s="2" t="n"/>
@@ -1003,7 +1003,7 @@
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t>Evalué si un fideicomiso u otra figura conviene para administrar los recursos de mi hij@.</t>
+          <t>Sé si yo (o el otro padre/madre) cotizo o coticé en el IMSS o el ISSSTE.</t>
         </is>
       </c>
       <c r="B44" s="13" t="n"/>
@@ -1014,7 +1014,7 @@
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>Definí quién administraría los recursos y bajo qué instrucciones.</t>
+          <t>Sé quién está designado como beneficiario en mi cuenta de AFORE.</t>
         </is>
       </c>
       <c r="B45" s="15" t="n"/>
@@ -1025,7 +1025,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>Las instrucciones reflejan las necesidades reales de mi hij@ (terapias, vivienda, salud).</t>
+          <t>Sé que un hij@ con discapacidad puede conservar una pensión por orfandad más allá de la edad habitual, conforme a la ley.</t>
         </is>
       </c>
       <c r="B46" s="13" t="n"/>
@@ -1036,7 +1036,7 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>Hay una persona de confianza que supervise esa administración.</t>
+          <t>Sé que los recursos de mi AFORE pueden pasar a mis beneficiarios o convertirse en pensión, conforme a la ley.</t>
         </is>
       </c>
       <c r="B47" s="15" t="n"/>
@@ -1044,70 +1044,70 @@
       <c r="D47" s="15" t="n"/>
       <c r="E47" s="15" t="n"/>
     </row>
-    <row r="49" ht="26" customHeight="1">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t>5. Red de apoyo</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="n"/>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="11" t="inlineStr">
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>Tengo identificados los requisitos y documentos para que mi hij@ pueda solicitar esa pensión o esos recursos.</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="n"/>
+      <c r="C48" s="13" t="n"/>
+      <c r="D48" s="13" t="n"/>
+      <c r="E48" s="13" t="n"/>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>Mi red de apoyo sabe que esa pensión / AFORE podría existir y a qué institución (IMSS, ISSSTE o Afore) acudir.</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="n"/>
+      <c r="C49" s="15" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="15" t="n"/>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>5. Fideicomiso o mecanismo de administración</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>Punto a revisar</t>
         </is>
       </c>
-      <c r="B50" s="11" t="inlineStr">
+      <c r="B52" s="11" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="C50" s="11" t="inlineStr">
+      <c r="C52" s="11" t="inlineStr">
         <is>
           <t>Riesgo detectado</t>
         </is>
       </c>
-      <c r="D50" s="11" t="inlineStr">
+      <c r="D52" s="11" t="inlineStr">
         <is>
           <t>Acción a tomar</t>
         </is>
       </c>
-      <c r="E50" s="11" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Fecha compromiso</t>
         </is>
       </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
-        <is>
-          <t>Identifiqué a las personas que cuidarían de mi hij@ (familiares, amigos, profesionales).</t>
-        </is>
-      </c>
-      <c r="B51" s="13" t="n"/>
-      <c r="C51" s="13" t="n"/>
-      <c r="D51" s="13" t="n"/>
-      <c r="E51" s="13" t="n"/>
-    </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="14" t="inlineStr">
-        <is>
-          <t>Esas personas saben y aceptaron esa responsabilidad.</t>
-        </is>
-      </c>
-      <c r="B52" s="15" t="n"/>
-      <c r="C52" s="15" t="n"/>
-      <c r="D52" s="15" t="n"/>
-      <c r="E52" s="15" t="n"/>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>La red no depende de una sola persona.</t>
+          <t>Evalué si un fideicomiso u otra figura conviene para administrar los recursos de mi hij@.</t>
         </is>
       </c>
       <c r="B53" s="13" t="n"/>
@@ -1118,7 +1118,7 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>Mi hij@ conoce y tiene relación con su red de apoyo.</t>
+          <t>Definí quién administraría los recursos y bajo qué instrucciones.</t>
         </is>
       </c>
       <c r="B54" s="15" t="n"/>
@@ -1126,70 +1126,70 @@
       <c r="D54" s="15" t="n"/>
       <c r="E54" s="15" t="n"/>
     </row>
-    <row r="56" ht="26" customHeight="1">
-      <c r="A56" s="8" t="inlineStr">
-        <is>
-          <t>6. Carta de intención</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="n"/>
-      <c r="C56" s="2" t="n"/>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="n"/>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>Las instrucciones reflejan las necesidades reales de mi hij@ (terapias, vivienda, salud).</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="n"/>
+      <c r="C55" s="13" t="n"/>
+      <c r="D55" s="13" t="n"/>
+      <c r="E55" s="13" t="n"/>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>Hay una persona de confianza que supervise esa administración.</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="n"/>
+      <c r="C56" s="15" t="n"/>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="15" t="n"/>
+    </row>
+    <row r="58" ht="26" customHeight="1">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>6. Red de apoyo</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="n"/>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>Punto a revisar</t>
         </is>
       </c>
-      <c r="B57" s="11" t="inlineStr">
+      <c r="B59" s="11" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="C57" s="11" t="inlineStr">
+      <c r="C59" s="11" t="inlineStr">
         <is>
           <t>Riesgo detectado</t>
         </is>
       </c>
-      <c r="D57" s="11" t="inlineStr">
+      <c r="D59" s="11" t="inlineStr">
         <is>
           <t>Acción a tomar</t>
         </is>
       </c>
-      <c r="E57" s="11" t="inlineStr">
+      <c r="E59" s="11" t="inlineStr">
         <is>
           <t>Fecha compromiso</t>
         </is>
       </c>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="12" t="inlineStr">
-        <is>
-          <t>Escribí una carta de intención con mis deseos sobre el cuidado de mi hij@.</t>
-        </is>
-      </c>
-      <c r="B58" s="13" t="n"/>
-      <c r="C58" s="13" t="n"/>
-      <c r="D58" s="13" t="n"/>
-      <c r="E58" s="13" t="n"/>
-    </row>
-    <row r="59" ht="30" customHeight="1">
-      <c r="A59" s="14" t="inlineStr">
-        <is>
-          <t>La carta describe a quién quiero que lo cuide y cómo.</t>
-        </is>
-      </c>
-      <c r="B59" s="15" t="n"/>
-      <c r="C59" s="15" t="n"/>
-      <c r="D59" s="15" t="n"/>
-      <c r="E59" s="15" t="n"/>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="12" t="inlineStr">
         <is>
-          <t>La carta está en un lugar conocido por mi red de apoyo.</t>
+          <t>Identifiqué a las personas que cuidarían de mi hij@ (familiares, amigos, profesionales).</t>
         </is>
       </c>
       <c r="B60" s="13" t="n"/>
@@ -1197,152 +1197,152 @@
       <c r="D60" s="13" t="n"/>
       <c r="E60" s="13" t="n"/>
     </row>
-    <row r="62" ht="26" customHeight="1">
-      <c r="A62" s="8" t="inlineStr">
-        <is>
-          <t>7. Documentación de cuidados</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="2" t="n"/>
-      <c r="D62" s="2" t="n"/>
-      <c r="E62" s="2" t="n"/>
-    </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="11" t="inlineStr">
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>Esas personas saben y aceptaron esa responsabilidad.</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="n"/>
+      <c r="C61" s="15" t="n"/>
+      <c r="D61" s="15" t="n"/>
+      <c r="E61" s="15" t="n"/>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="12" t="inlineStr">
+        <is>
+          <t>La red no depende de una sola persona.</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="n"/>
+      <c r="C62" s="13" t="n"/>
+      <c r="D62" s="13" t="n"/>
+      <c r="E62" s="13" t="n"/>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>Mi hij@ conoce y tiene relación con su red de apoyo.</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="n"/>
+      <c r="C63" s="15" t="n"/>
+      <c r="D63" s="15" t="n"/>
+      <c r="E63" s="15" t="n"/>
+    </row>
+    <row r="65" ht="26" customHeight="1">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>7. Carta de intención</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="n"/>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="11" t="inlineStr">
         <is>
           <t>Punto a revisar</t>
         </is>
       </c>
-      <c r="B63" s="11" t="inlineStr">
+      <c r="B66" s="11" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="C63" s="11" t="inlineStr">
+      <c r="C66" s="11" t="inlineStr">
         <is>
           <t>Riesgo detectado</t>
         </is>
       </c>
-      <c r="D63" s="11" t="inlineStr">
+      <c r="D66" s="11" t="inlineStr">
         <is>
           <t>Acción a tomar</t>
         </is>
       </c>
-      <c r="E63" s="11" t="inlineStr">
+      <c r="E66" s="11" t="inlineStr">
         <is>
           <t>Fecha compromiso</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="12" t="inlineStr">
-        <is>
-          <t>Documenté rutinas, hábitos y preferencias de mi hij@.</t>
-        </is>
-      </c>
-      <c r="B64" s="13" t="n"/>
-      <c r="C64" s="13" t="n"/>
-      <c r="D64" s="13" t="n"/>
-      <c r="E64" s="13" t="n"/>
-    </row>
-    <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="14" t="inlineStr">
-        <is>
-          <t>Documenté tratamientos, terapias y medicamentos actuales.</t>
-        </is>
-      </c>
-      <c r="B65" s="15" t="n"/>
-      <c r="C65" s="15" t="n"/>
-      <c r="D65" s="15" t="n"/>
-      <c r="E65" s="15" t="n"/>
-    </row>
-    <row r="66" ht="30" customHeight="1">
-      <c r="A66" s="12" t="inlineStr">
-        <is>
-          <t>Documenté contactos de médicos, terapeutas e instituciones.</t>
-        </is>
-      </c>
-      <c r="B66" s="13" t="n"/>
-      <c r="C66" s="13" t="n"/>
-      <c r="D66" s="13" t="n"/>
-      <c r="E66" s="13" t="n"/>
-    </row>
     <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="14" t="inlineStr">
-        <is>
-          <t>La documentación está accesible para quienes cuidarían de mi hij@.</t>
-        </is>
-      </c>
-      <c r="B67" s="15" t="n"/>
-      <c r="C67" s="15" t="n"/>
-      <c r="D67" s="15" t="n"/>
-      <c r="E67" s="15" t="n"/>
-    </row>
-    <row r="69" ht="26" customHeight="1">
-      <c r="A69" s="8" t="inlineStr">
-        <is>
-          <t>8. Señales de alerta — ¿detectas alguno de estos focos rojos?</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="n"/>
-      <c r="C69" s="2" t="n"/>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="n"/>
-    </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="11" t="inlineStr">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>Escribí una carta de intención con mis deseos sobre el cuidado de mi hij@.</t>
+        </is>
+      </c>
+      <c r="B67" s="13" t="n"/>
+      <c r="C67" s="13" t="n"/>
+      <c r="D67" s="13" t="n"/>
+      <c r="E67" s="13" t="n"/>
+    </row>
+    <row r="68" ht="30" customHeight="1">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>La carta describe a quién quiero que lo cuide y cómo.</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="n"/>
+      <c r="C68" s="15" t="n"/>
+      <c r="D68" s="15" t="n"/>
+      <c r="E68" s="15" t="n"/>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t>La carta está en un lugar conocido por mi red de apoyo.</t>
+        </is>
+      </c>
+      <c r="B69" s="13" t="n"/>
+      <c r="C69" s="13" t="n"/>
+      <c r="D69" s="13" t="n"/>
+      <c r="E69" s="13" t="n"/>
+    </row>
+    <row r="71" ht="26" customHeight="1">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>8. Documentación de cuidados</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="n"/>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="11" t="inlineStr">
         <is>
           <t>Punto a revisar</t>
         </is>
       </c>
-      <c r="B70" s="11" t="inlineStr">
+      <c r="B72" s="11" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="C70" s="11" t="inlineStr">
+      <c r="C72" s="11" t="inlineStr">
         <is>
           <t>Riesgo detectado</t>
         </is>
       </c>
-      <c r="D70" s="11" t="inlineStr">
+      <c r="D72" s="11" t="inlineStr">
         <is>
           <t>Acción a tomar</t>
         </is>
       </c>
-      <c r="E70" s="11" t="inlineStr">
+      <c r="E72" s="11" t="inlineStr">
         <is>
           <t>Fecha compromiso</t>
         </is>
       </c>
-    </row>
-    <row r="71" ht="30" customHeight="1">
-      <c r="A71" s="12" t="inlineStr">
-        <is>
-          <t>Si yo faltara mañana, no hay una persona claramente definida para cuidar de mi hij@.</t>
-        </is>
-      </c>
-      <c r="B71" s="13" t="n"/>
-      <c r="C71" s="13" t="n"/>
-      <c r="D71" s="13" t="n"/>
-      <c r="E71" s="13" t="n"/>
-    </row>
-    <row r="72" ht="30" customHeight="1">
-      <c r="A72" s="14" t="inlineStr">
-        <is>
-          <t>No sé si los recursos alcanzarían para sostener su calidad de vida.</t>
-        </is>
-      </c>
-      <c r="B72" s="15" t="n"/>
-      <c r="C72" s="15" t="n"/>
-      <c r="D72" s="15" t="n"/>
-      <c r="E72" s="15" t="n"/>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="12" t="inlineStr">
         <is>
-          <t>No hay instrucciones por escrito para quienes se queden a cargo.</t>
+          <t>Documenté rutinas, hábitos y preferencias de mi hij@.</t>
         </is>
       </c>
       <c r="B73" s="13" t="n"/>
@@ -1353,7 +1353,7 @@
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="14" t="inlineStr">
         <is>
-          <t>Estoy confiando solo en la buena voluntad de la familia.</t>
+          <t>Documenté tratamientos, terapias y medicamentos actuales.</t>
         </is>
       </c>
       <c r="B74" s="15" t="n"/>
@@ -1364,7 +1364,7 @@
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t>Nunca calculé el costo real de los cuidados a largo plazo.</t>
+          <t>Documenté contactos de médicos, terapeutas e instituciones.</t>
         </is>
       </c>
       <c r="B75" s="13" t="n"/>
@@ -1372,118 +1372,223 @@
       <c r="D75" s="13" t="n"/>
       <c r="E75" s="13" t="n"/>
     </row>
-    <row r="77" ht="26" customHeight="1">
-      <c r="A77" s="8" t="inlineStr">
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <t>La documentación está accesible para quienes cuidarían de mi hij@.</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="n"/>
+      <c r="C76" s="15" t="n"/>
+      <c r="D76" s="15" t="n"/>
+      <c r="E76" s="15" t="n"/>
+    </row>
+    <row r="78" ht="26" customHeight="1">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>9. Señales de alerta — ¿detectas alguno de estos focos rojos?</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n"/>
+      <c r="C78" s="2" t="n"/>
+      <c r="D78" s="2" t="n"/>
+      <c r="E78" s="2" t="n"/>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t>Punto a revisar</t>
+        </is>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="inlineStr">
+        <is>
+          <t>Riesgo detectado</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>Acción a tomar</t>
+        </is>
+      </c>
+      <c r="E79" s="11" t="inlineStr">
+        <is>
+          <t>Fecha compromiso</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="12" t="inlineStr">
+        <is>
+          <t>Si yo faltara mañana, no hay una persona claramente definida para cuidar de mi hij@.</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="n"/>
+      <c r="C80" s="13" t="n"/>
+      <c r="D80" s="13" t="n"/>
+      <c r="E80" s="13" t="n"/>
+    </row>
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>No sé si los recursos alcanzarían para sostener su calidad de vida.</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="n"/>
+      <c r="C81" s="15" t="n"/>
+      <c r="D81" s="15" t="n"/>
+      <c r="E81" s="15" t="n"/>
+    </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="12" t="inlineStr">
+        <is>
+          <t>No hay instrucciones por escrito para quienes se queden a cargo.</t>
+        </is>
+      </c>
+      <c r="B82" s="13" t="n"/>
+      <c r="C82" s="13" t="n"/>
+      <c r="D82" s="13" t="n"/>
+      <c r="E82" s="13" t="n"/>
+    </row>
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>Estoy confiando solo en la buena voluntad de la familia.</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="n"/>
+      <c r="C83" s="15" t="n"/>
+      <c r="D83" s="15" t="n"/>
+      <c r="E83" s="15" t="n"/>
+    </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="12" t="inlineStr">
+        <is>
+          <t>Nunca calculé el costo real de los cuidados a largo plazo.</t>
+        </is>
+      </c>
+      <c r="B84" s="13" t="n"/>
+      <c r="C84" s="13" t="n"/>
+      <c r="D84" s="13" t="n"/>
+      <c r="E84" s="13" t="n"/>
+    </row>
+    <row r="86" ht="26" customHeight="1">
+      <c r="A86" s="8" t="inlineStr">
         <is>
           <t>¿Cada cuándo revisar?</t>
         </is>
       </c>
-      <c r="B77" s="2" t="n"/>
-      <c r="C77" s="2" t="n"/>
-      <c r="D77" s="2" t="n"/>
-      <c r="E77" s="2" t="n"/>
-    </row>
-    <row r="78" ht="15" customHeight="1">
-      <c r="A78" s="7" t="inlineStr">
+      <c r="B86" s="2" t="n"/>
+      <c r="C86" s="2" t="n"/>
+      <c r="D86" s="2" t="n"/>
+      <c r="E86" s="2" t="n"/>
+    </row>
+    <row r="87" ht="15" customHeight="1">
+      <c r="A87" s="7" t="inlineStr">
         <is>
           <t>•  Cambios en la condición o necesidades de tu hij@</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="15" customHeight="1">
-      <c r="A79" s="7" t="inlineStr">
+    <row r="88" ht="15" customHeight="1">
+      <c r="A88" s="7" t="inlineStr">
         <is>
           <t>•  Matrimonio, divorcio o nacimiento de otros hijos</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="15" customHeight="1">
-      <c r="A80" s="7" t="inlineStr">
+    <row r="89" ht="15" customHeight="1">
+      <c r="A89" s="7" t="inlineStr">
         <is>
           <t>•  Cambio importante de patrimonio</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="15" customHeight="1">
-      <c r="A81" s="7" t="inlineStr">
+    <row r="90" ht="15" customHeight="1">
+      <c r="A90" s="7" t="inlineStr">
         <is>
           <t>•  Contratación de nuevas pólizas o cambio de asesor</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="15" customHeight="1">
-      <c r="A82" s="7" t="inlineStr">
+    <row r="91" ht="15" customHeight="1">
+      <c r="A91" s="7" t="inlineStr">
         <is>
           <t>•  Al menos una vez al año, aunque no haya cambios</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="26" customHeight="1">
-      <c r="A84" s="8" t="inlineStr">
+    <row r="93" ht="26" customHeight="1">
+      <c r="A93" s="8" t="inlineStr">
         <is>
           <t>Empieza hoy</t>
         </is>
       </c>
-      <c r="B84" s="2" t="n"/>
-      <c r="C84" s="2" t="n"/>
-      <c r="D84" s="2" t="n"/>
-      <c r="E84" s="2" t="n"/>
-    </row>
-    <row r="85" ht="58" customHeight="1">
-      <c r="A85" s="16" t="inlineStr">
+      <c r="B93" s="2" t="n"/>
+      <c r="C93" s="2" t="n"/>
+      <c r="D93" s="2" t="n"/>
+      <c r="E93" s="2" t="n"/>
+    </row>
+    <row r="94" ht="58" customHeight="1">
+      <c r="A94" s="16" t="inlineStr">
         <is>
           <t>No necesitas ser millonario ni tenerlo todo resuelto. Lo que tu hij@ necesita es claridad: quién lo cuidará, cómo se administrarán los recursos y qué pasará cuando tú ya no estés para decidir. Empezar hoy vale más que el plan perfecto que nunca llega.</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="24" customHeight="1">
-      <c r="A87" s="17" t="inlineStr">
+    <row r="96" ht="24" customHeight="1">
+      <c r="A96" s="17" t="inlineStr">
         <is>
           <t>¿Quieres ordenar tu plan con acompañamiento? Agenda una sesión inicial.  ·  iriatalan.com.mx</t>
         </is>
       </c>
-      <c r="B87" s="4" t="n"/>
-      <c r="C87" s="4" t="n"/>
-      <c r="D87" s="4" t="n"/>
-      <c r="E87" s="4" t="n"/>
+      <c r="B96" s="4" t="n"/>
+      <c r="C96" s="4" t="n"/>
+      <c r="D96" s="4" t="n"/>
+      <c r="E96" s="4" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="A77:E77"/>
-    <mergeCell ref="A82:E82"/>
+  <mergeCells count="33">
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="B15:E15"/>
-    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A51:E51"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A94:E94"/>
     <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A79:E79"/>
-    <mergeCell ref="A69:E69"/>
+    <mergeCell ref="A88:E88"/>
     <mergeCell ref="A87:E87"/>
+    <mergeCell ref="A65:E65"/>
     <mergeCell ref="A78:E78"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A90:E90"/>
     <mergeCell ref="B16:E16"/>
-    <mergeCell ref="A84:E84"/>
-    <mergeCell ref="A80:E80"/>
-    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A89:E89"/>
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A86:E86"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="A42:E42"/>
-    <mergeCell ref="A85:E85"/>
+    <mergeCell ref="A71:E71"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="B14:E14"/>
+    <mergeCell ref="A91:E91"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A62:E62"/>
-    <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A96:E96"/>
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A58:E58"/>
     <mergeCell ref="A9:E9"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B21 B22 B23 B24 B25 B29 B30 B31 B32 B33 B37 B38 B39 B40 B44 B45 B46 B47 B51 B52 B53 B54 B58 B59 B60 B64 B65 B66 B67 B71 B72 B73 B74 B75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B21 B22 B23 B24 B25 B29 B30 B31 B32 B33 B37 B38 B39 B40 B44 B45 B46 B47 B48 B49 B53 B54 B55 B56 B60 B61 B62 B63 B67 B68 B69 B73 B74 B75 B76 B80 B81 B82 B83 B84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Resuelto,Pendiente,No estoy seguro(a),No aplica"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>